<commit_message>
update skills and assest
</commit_message>
<xml_diff>
--- a/assets/year-2026/event-plan-2026.xlsx
+++ b/assets/year-2026/event-plan-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/paolorossi/Develop/firefighter-app-ui/assets/year-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D942705-664A-9D47-8100-81D2C31E0737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14B15997-D8BE-A04E-BAE5-25ED58F12E25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="38400" windowHeight="20980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="130">
   <si>
     <t>id</t>
   </si>
@@ -326,9 +326,6 @@
   </si>
   <si>
     <t>nachtdienst-2026-12-07</t>
-  </si>
-  <si>
-    <t>burger.franz;oberhollenzer.christoph;mair.stefan;rossi.paolo</t>
   </si>
   <si>
     <t>nachtdienst-2026-12-08</t>
@@ -2278,7 +2275,7 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J56" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.2">
@@ -2304,7 +2301,7 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J57" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.2">
@@ -2330,7 +2327,7 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J58" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.2">
@@ -2356,7 +2353,7 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J59" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.2">
@@ -2382,7 +2379,7 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J60" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.2">
@@ -2408,7 +2405,7 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J61" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.2">
@@ -2434,7 +2431,7 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J62" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.2">
@@ -2850,12 +2847,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J78" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B79" t="s">
         <v>11</v>
@@ -2876,12 +2873,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J79" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B80" t="s">
         <v>11</v>
@@ -2902,12 +2899,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J80" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B81" t="s">
         <v>11</v>
@@ -2928,12 +2925,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J81" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A82" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B82" s="8" t="s">
         <v>24</v>
@@ -2961,7 +2958,7 @@
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B83" t="s">
         <v>11</v>
@@ -2982,12 +2979,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J83" s="3" t="s">
-        <v>102</v>
+        <v>128</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B84" t="s">
         <v>11</v>
@@ -3008,12 +3005,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J84" s="3" t="s">
-        <v>102</v>
+        <v>128</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B85" t="s">
         <v>11</v>
@@ -3034,12 +3031,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J85" s="3" t="s">
-        <v>102</v>
+        <v>128</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A86" s="12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B86" s="12" t="s">
         <v>66</v>
@@ -3067,7 +3064,7 @@
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B87" t="s">
         <v>11</v>
@@ -3088,12 +3085,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J87" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B88" t="s">
         <v>11</v>
@@ -3114,12 +3111,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J88" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B89" t="s">
         <v>11</v>
@@ -3140,12 +3137,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J89" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B90" t="s">
         <v>11</v>
@@ -3166,12 +3163,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J90" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B91" t="s">
         <v>11</v>
@@ -3192,15 +3189,15 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J91" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A92" s="16" t="s">
+        <v>116</v>
+      </c>
+      <c r="B92" s="16" t="s">
         <v>117</v>
-      </c>
-      <c r="B92" s="16" t="s">
-        <v>118</v>
       </c>
       <c r="C92" s="16" t="b">
         <v>1</v>
@@ -3219,7 +3216,7 @@
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B93" t="s">
         <v>11</v>
@@ -3240,12 +3237,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J93" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B94" t="s">
         <v>11</v>
@@ -3266,12 +3263,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J94" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B95" t="s">
         <v>11</v>
@@ -3292,12 +3289,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J95" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B96" t="s">
         <v>11</v>
@@ -3318,12 +3315,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J96" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B97" t="s">
         <v>11</v>
@@ -3344,12 +3341,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J97" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B98" t="s">
         <v>11</v>
@@ -3370,12 +3367,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J98" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B99" t="s">
         <v>11</v>
@@ -3396,12 +3393,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J99" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B100" t="s">
         <v>11</v>
@@ -3422,12 +3419,12 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J100" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B101" t="s">
         <v>11</v>
@@ -3448,7 +3445,7 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J101" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>